<commit_message>
cambios para convalidar al español
</commit_message>
<xml_diff>
--- a/output/StructureDefinition-BundleMhd.xlsx
+++ b/output/StructureDefinition-BundleMhd.xlsx
@@ -27,13 +27,13 @@
     <t>URL</t>
   </si>
   <si>
-    <t>http://mhd.ri.hsisalud.org/StructureDefinition/BundleMhd</t>
+    <t>https://hl7chile.cl/fhir/ig/mhd/StructureDefinition/BundleMhd</t>
   </si>
   <si>
     <t>Version</t>
   </si>
   <si>
-    <t>0.3.0</t>
+    <t>0.1.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,25 +57,25 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-22</t>
+    <t>2026-10-14</t>
   </si>
   <si>
     <t>Publisher</t>
   </si>
   <si>
-    <t>HSI Pladema</t>
+    <t>Hl7 Chile</t>
   </si>
   <si>
     <t>Contact</t>
   </si>
   <si>
-    <t>HSI Pladema (https://hsi.pladema.net)</t>
+    <t>Hl7 Chile (https://hl7chile.cl/)</t>
   </si>
   <si>
     <t>Jurisdiction</t>
   </si>
   <si>
-    <t>Argentina</t>
+    <t>Chile</t>
   </si>
   <si>
     <t>Description</t>
@@ -433,7 +433,7 @@
     <t>Bundle.meta.profile</t>
   </si>
   <si>
-    <t xml:space="preserve">canonical(StructureDefinition)
+    <t xml:space="preserve">canonical(StructureDefinition|4.0.1)
 </t>
   </si>
   <si>
@@ -468,7 +468,7 @@
     <t>Security Labels from the Healthcare Privacy and Security Classification System.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/security-labels</t>
+    <t>http://hl7.org/fhir/ValueSet/security-labels|4.0.1</t>
   </si>
   <si>
     <t>Meta.security</t>
@@ -492,7 +492,7 @@
     <t>Codes that represent various types of tags, commonly workflow-related; e.g. "Needs review by Dr. Jones".</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/common-tags</t>
+    <t>http://hl7.org/fhir/ValueSet/common-tags|4.0.1</t>
   </si>
   <si>
     <t>Meta.tag</t>
@@ -535,7 +535,7 @@
     <t>A human language.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/languages</t>
+    <t>http://hl7.org/fhir/ValueSet/languages|4.0.1</t>
   </si>
   <si>
     <t>Resource.language</t>
@@ -1016,7 +1016,7 @@
 WorkingListOrganizer</t>
   </si>
   <si>
-    <t xml:space="preserve">List {http://mhd.ri.hsisalud.org/StructureDefinition/ListMhd}
+    <t xml:space="preserve">List {https://hl7chile.cl/fhir/ig/mhd/StructureDefinition/ListMhd}
 </t>
   </si>
   <si>
@@ -1140,7 +1140,7 @@
     <t>Bundle.entry:DocumentRefs.resource</t>
   </si>
   <si>
-    <t xml:space="preserve">DocumentReference {http://mhd.ri.hsisalud.org/StructureDefinition/ReferenciaDocumental}
+    <t xml:space="preserve">DocumentReference {https://hl7chile.cl/fhir/ig/mhd/StructureDefinition/ReferenciaDocumental}
 </t>
   </si>
   <si>
@@ -1195,7 +1195,7 @@
     <t>Bundle.entry:DocumentRefs.request.url</t>
   </si>
   <si>
-    <t>/DocumentReference</t>
+    <t>DocumentReference</t>
   </si>
   <si>
     <t>Bundle.entry:DocumentRefs.request.ifNoneMatch</t>
@@ -1246,7 +1246,7 @@
     <t>the superseded DocumentReference resources</t>
   </si>
   <si>
-    <t>any updated DocumentReference that are part of the SubmissionSet if a new new DocumentReference replaces this DocumentReference.</t>
+    <t>any updated DocumentReference that are part of the SubmissionSet if a new DocumentReference replaces this DocumentReference.</t>
   </si>
   <si>
     <t>Bundle.entry:UpdateDocumentRefs.id</t>
@@ -1512,7 +1512,7 @@
     <t>Bundle.entry:FhirDocuments.resource</t>
   </si>
   <si>
-    <t xml:space="preserve">Bundle {http://ips.ri.hsisalud.org/StructureDefinition/BundleDocArg}
+    <t xml:space="preserve">Bundle {Bundle}
 </t>
   </si>
   <si>
@@ -1731,7 +1731,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Patient {http://ips.ri.hsisalud.org/StructureDefinition/PacienteArg}
+    <t xml:space="preserve">Patient {https://hl7chile.cl/fhir/ig/clcore/StructureDefinition/CorePacienteCl}
 </t>
   </si>
   <si>
@@ -2162,17 +2162,17 @@
   <dimension ref="A1:AN281"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="52.5" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="34.23828125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="18.6640625" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="4" max="4" width="24.95703125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="5" max="5" width="5.29296875" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="4.21484375" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="4.55078125" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="13.1171875" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="10.75390625" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="51.23828125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="33.44140625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="18.16015625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="4" max="4" width="24.67578125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="4.65625" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="76.890625" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="76.31640625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -2181,26 +2181,26 @@
     <col min="17" max="17" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="18" max="18" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="19" max="19" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="20" max="20" width="48.1484375" customWidth="true" bestFit="true"/>
-    <col min="21" max="21" width="14.08984375" customWidth="true" bestFit="true"/>
-    <col min="22" max="22" width="14.4296875" customWidth="true" bestFit="true"/>
-    <col min="23" max="23" width="15.31640625" customWidth="true" bestFit="true"/>
-    <col min="24" max="24" width="14.62890625" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="146.4296875" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="57.4921875" customWidth="true" bestFit="true"/>
-    <col min="27" max="27" width="5.10546875" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="19.375" customWidth="true" bestFit="true"/>
-    <col min="29" max="29" width="43.54296875" customWidth="true" bestFit="true"/>
-    <col min="30" max="30" width="13.44140625" customWidth="true" bestFit="true"/>
-    <col min="31" max="31" width="11.03515625" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="31.015625" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="33" max="33" width="8.51953125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="34" max="34" width="8.859375" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" width="48.48046875" customWidth="true" bestFit="true"/>
+    <col min="21" max="21" width="14.72265625" customWidth="true" bestFit="true"/>
+    <col min="22" max="22" width="15.13671875" customWidth="true" bestFit="true"/>
+    <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
+    <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="144.1953125" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="54.09765625" customWidth="true" bestFit="true"/>
+    <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
+    <col min="29" max="29" width="42.89453125" customWidth="true" bestFit="true"/>
+    <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
+    <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="29.98828125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
-    <col min="37" max="37" width="22.43359375" customWidth="true" bestFit="true"/>
-    <col min="38" max="38" width="43.1796875" customWidth="true" bestFit="true"/>
-    <col min="39" max="39" width="37.16015625" customWidth="true" bestFit="true"/>
-    <col min="40" max="40" width="29.45703125" customWidth="true" bestFit="true"/>
+    <col min="37" max="37" width="24.1328125" customWidth="true" bestFit="true"/>
+    <col min="38" max="38" width="42.9375" customWidth="true" bestFit="true"/>
+    <col min="39" max="39" width="36.84375" customWidth="true" bestFit="true"/>
+    <col min="40" max="40" width="31.65234375" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4956,7 +4956,7 @@
         <v>78</v>
       </c>
       <c r="H25" t="s" s="2">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="I25" t="s" s="2">
         <v>76</v>
@@ -5617,7 +5617,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
         <v>233</v>
       </c>
@@ -5636,7 +5636,7 @@
         <v>86</v>
       </c>
       <c r="H31" t="s" s="2">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="I31" t="s" s="2">
         <v>76</v>

</xml_diff>